<commit_message>
Rental tracker v1.2: polished dashboard, error highlighting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dl/QkFNAj8Wx9bU9aQs/Rental-Property-Tracker-NoraStudio.xlsx
+++ b/dl/QkFNAj8Wx9bU9aQs/Rental-Property-Tracker-NoraStudio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\Joker\projects\products\01-rental-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714F6372-65AC-4386-8AF0-B3BA8734C4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E34B1B-04B4-4D90-884E-B40123A4CD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34290" yWindow="-210" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="140">
   <si>
     <t>Rental Property Tracker</t>
   </si>
@@ -120,6 +120,9 @@
     <t>Net income</t>
   </si>
   <si>
+    <t>Sort key</t>
+  </si>
+  <si>
     <t>CASH FLOW (NO DEPR.)</t>
   </si>
   <si>
@@ -183,6 +186,12 @@
     <t>Amount</t>
   </si>
   <si>
+    <t>Top expenses</t>
+  </si>
+  <si>
+    <t>Property (sorted)</t>
+  </si>
+  <si>
     <t>Properties</t>
   </si>
   <si>
@@ -226,6 +235,9 @@
   </si>
   <si>
     <t>One row per payment. Amounts are always positive; the Type column works out income vs. expense.</t>
+  </si>
+  <si>
+    <t>Red cell = missing date, property or category; that row is left out of the totals until fixed.</t>
   </si>
   <si>
     <t>Date</t>
@@ -458,7 +470,7 @@
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00;\(\$#,##0.00\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -507,6 +519,12 @@
       <i/>
       <sz val="9"/>
       <color rgb="FF666666"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFB03A2E"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -608,7 +626,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -629,42 +647,44 @@
     <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFBE0B8"/>
+          <bgColor rgb="FFFBE0B8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -672,6 +692,31 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8C9C4"/>
+          <bgColor rgb="FFF8C9C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8C9C4"/>
+          <bgColor rgb="FFF8C9C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8C9C4"/>
+          <bgColor rgb="FFF8C9C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8C9C4"/>
+          <bgColor rgb="FFF8C9C4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -836,7 +881,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D496-4D7D-A9DA-98FADD68BE1C}"/>
+              <c16:uniqueId val="{00000000-E003-4570-B6C7-9108F0A37CEB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -957,7 +1002,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D496-4D7D-A9DA-98FADD68BE1C}"/>
+              <c16:uniqueId val="{00000001-E003-4570-B6C7-9108F0A37CEB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1041,7 +1086,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Expenses by category</a:t>
+              <a:t>Top expenses by category</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1060,7 +1105,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!$W$33</c:f>
+              <c:f>Dashboard!$W$52</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1083,71 +1128,35 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$V$34:$V$48</c:f>
+              <c:f>Dashboard!$V$53:$V$60</c:f>
               <c:strCache>
-                <c:ptCount val="15"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Advertising</c:v>
+                  <c:v>Depreciation (estimated)</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Auto and travel</c:v>
+                  <c:v>Mortgage interest paid to banks</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Cleaning and maintenance</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Commissions</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Insurance</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Legal and other professional fees</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Management fees</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Mortgage interest paid to banks</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Other interest</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>Repairs</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Supplies</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Taxes</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>Utilities</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>Other</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>Depreciation (estimated)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$W$34:$W$48</c:f>
+              <c:f>Dashboard!$W$53:$W$60</c:f>
               <c:numCache>
                 <c:formatCode>\$#,##0.00;\(\$#,##0.00\);"-"</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>8181.82</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>215</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1162,35 +1171,14 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>612.4</c:v>
-                </c:pt>
-                <c:pt idx="8">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>215</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>8181.818181818182</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5957-4C12-B45E-5ACC1355024C}"/>
+              <c16:uniqueId val="{00000000-8B9A-44AE-8065-8A456071C59A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1209,7 +1197,7 @@
       <c:catAx>
         <c:axId val="10"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1232,12 +1220,12 @@
         <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:majorGridlines/>
-        <c:numFmt formatCode="\$#,##0" sourceLinked="0"/>
+        <c:numFmt formatCode="\$#,##0,&quot;K&quot;" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="10"/>
-        <c:crosses val="autoZero"/>
+        <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
@@ -1289,7 +1277,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!$W$4</c:f>
+              <c:f>Dashboard!$W$62</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1312,7 +1300,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$V$5:$V$14</c:f>
+              <c:f>Dashboard!$V$63:$V$72</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1323,12 +1311,12 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$W$5:$W$14</c:f>
+              <c:f>Dashboard!$W$63:$W$72</c:f>
               <c:numCache>
                 <c:formatCode>\$#,##0.00;\(\$#,##0.00\);"-"</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>-7559.2181818181816</c:v>
+                  <c:v>-7559.22</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1362,7 +1350,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5DCE-4535-A672-E676521EB8C0}"/>
+              <c16:uniqueId val="{00000000-6637-4558-85FD-33BE6D44ABAC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1381,14 +1369,14 @@
       <c:catAx>
         <c:axId val="10"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="low"/>
         <c:crossAx val="100"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -1409,7 +1397,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="10"/>
-        <c:crosses val="autoZero"/>
+        <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
@@ -1573,7 +1561,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C698-46E9-8E82-040E5D575B26}"/>
+              <c16:uniqueId val="{00000000-27CF-4B03-B4D9-AAA67948F477}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1599,7 +1587,7 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="low"/>
         <c:crossAx val="100"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -1778,7 +1766,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3614-4CF9-844E-E654E2F5B5E4}"/>
+              <c16:uniqueId val="{00000000-939C-4337-80B9-C97FAE101E61}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1893,7 +1881,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3614-4CF9-844E-E654E2F5B5E4}"/>
+              <c16:uniqueId val="{00000001-939C-4337-80B9-C97FAE101E61}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2540,7 +2528,7 @@
   <sheetPr>
     <tabColor rgb="FF5B3A86"/>
   </sheetPr>
-  <dimension ref="B1:Y48"/>
+  <dimension ref="B1:Y72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -2548,70 +2536,73 @@
     <col min="22" max="25" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="23" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:24" ht="23" x14ac:dyDescent="0.5">
       <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="str">
         <f>"Tax year "&amp;'Schedule E Summary'!C3&amp;"  |  updates automatically from your Transactions"</f>
         <v>Tax year 2026  |  updates automatically from your Transactions</v>
       </c>
     </row>
-    <row r="3" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:24" x14ac:dyDescent="0.35">
       <c r="V3" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B4" s="31" t="s">
+    <row r="4" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="B4" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="G4" s="31" t="s">
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="G4" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="L4" s="31" t="s">
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="L4" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
       <c r="V4" t="s">
         <v>24</v>
       </c>
       <c r="W4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B5" s="29">
+      <c r="X4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="B5" s="30">
         <f>'Schedule E Summary'!M24</f>
         <v>1450</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="G5" s="29">
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="G5" s="30">
         <f>'Schedule E Summary'!M25</f>
         <v>9009.2181818181816</v>
       </c>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="L5" s="29">
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="L5" s="30">
         <f>'Schedule E Summary'!M26</f>
         <v>-7559.2181818181816</v>
       </c>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
       <c r="V5" t="str">
         <f>IF(Properties!B5="","",Properties!B5)</f>
         <v>EXAMPLE: 412 Maple St (duplex)</v>
@@ -2620,20 +2611,24 @@
         <f>IF(Properties!B5="",0,'Schedule E Summary'!C26)</f>
         <v>-7559.2181818181816</v>
       </c>
-    </row>
-    <row r="6" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="30"/>
-      <c r="O6" s="30"/>
+      <c r="X5">
+        <f>IF(V5="",-1000000000000,W5)+20/1000000</f>
+        <v>-7559.2181618181812</v>
+      </c>
+    </row>
+    <row r="6" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="31"/>
       <c r="V6" t="str">
         <f>IF(Properties!B6="","",Properties!B6)</f>
         <v/>
@@ -2642,8 +2637,12 @@
         <f>IF(Properties!B6="",0,'Schedule E Summary'!D26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.35">
+      <c r="X6">
+        <f>IF(V6="",-1000000000000,W6)+19/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.35">
       <c r="V7" t="str">
         <f>IF(Properties!B7="","",Properties!B7)</f>
         <v/>
@@ -2652,26 +2651,30 @@
         <f>IF(Properties!B7="",0,'Schedule E Summary'!E26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B8" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="G8" s="31" t="s">
+      <c r="X7">
+        <f>IF(V7="",-1000000000000,W7)+18/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="B8" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="L8" s="31" t="s">
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="G8" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31"/>
+      <c r="L8" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
+      <c r="O8" s="31"/>
       <c r="V8" t="str">
         <f>IF(Properties!B8="","",Properties!B8)</f>
         <v/>
@@ -2680,29 +2683,33 @@
         <f>IF(Properties!B8="",0,'Schedule E Summary'!F26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B9" s="29">
+      <c r="X8">
+        <f>IF(V8="",-1000000000000,W8)+17/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="B9" s="30">
         <f>'Schedule E Summary'!M24-('Schedule E Summary'!M25-'Schedule E Summary'!M22)</f>
         <v>622.60000000000036</v>
       </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="G9" s="29">
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="G9" s="30">
         <f>'Rent Roll'!E66</f>
         <v>1450</v>
       </c>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="L9" s="32">
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="L9" s="33">
         <f>COUNTA(Properties!B5:B14)</f>
         <v>1</v>
       </c>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
       <c r="V9" t="str">
         <f>IF(Properties!B9="","",Properties!B9)</f>
         <v/>
@@ -2711,20 +2718,24 @@
         <f>IF(Properties!B9="",0,'Schedule E Summary'!G26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
+      <c r="X9">
+        <f>IF(V9="",-1000000000000,W9)+16/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.35">
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
+      <c r="O10" s="31"/>
       <c r="V10" t="str">
         <f>IF(Properties!B10="","",Properties!B10)</f>
         <v/>
@@ -2733,8 +2744,12 @@
         <f>IF(Properties!B10="",0,'Schedule E Summary'!H26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.35">
+      <c r="X10">
+        <f>IF(V10="",-1000000000000,W10)+15/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.35">
       <c r="V11" t="str">
         <f>IF(Properties!B11="","",Properties!B11)</f>
         <v/>
@@ -2743,8 +2758,12 @@
         <f>IF(Properties!B11="",0,'Schedule E Summary'!I26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.35">
+      <c r="X11">
+        <f>IF(V11="",-1000000000000,W11)+14/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.35">
       <c r="V12" t="str">
         <f>IF(Properties!B12="","",Properties!B12)</f>
         <v/>
@@ -2753,8 +2772,12 @@
         <f>IF(Properties!B12="",0,'Schedule E Summary'!J26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.35">
+      <c r="X12">
+        <f>IF(V12="",-1000000000000,W12)+13/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.35">
       <c r="V13" t="str">
         <f>IF(Properties!B13="","",Properties!B13)</f>
         <v/>
@@ -2763,8 +2786,12 @@
         <f>IF(Properties!B13="",0,'Schedule E Summary'!K26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.35">
+      <c r="X13">
+        <f>IF(V13="",-1000000000000,W13)+12/1000000</f>
+        <v>-1000000000000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:24" x14ac:dyDescent="0.35">
       <c r="V14" t="str">
         <f>IF(Properties!B14="","",Properties!B14)</f>
         <v/>
@@ -2773,31 +2800,35 @@
         <f>IF(Properties!B14="",0,'Schedule E Summary'!L26)</f>
         <v>0</v>
       </c>
+      <c r="X14">
+        <f>IF(V14="",-1000000000000,W14)+11/1000000</f>
+        <v>-1000000000000</v>
+      </c>
     </row>
     <row r="17" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Y17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="W18" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,1)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,1)</f>
         <v>1450</v>
       </c>
       <c r="X18" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,1)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,1)</f>
         <v>827.4</v>
       </c>
       <c r="Y18" s="6">
@@ -2807,14 +2838,14 @@
     </row>
     <row r="19" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W19" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,2)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,2)</f>
         <v>0</v>
       </c>
       <c r="X19" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,2)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,2)</f>
         <v>0</v>
       </c>
       <c r="Y19" s="6">
@@ -2824,14 +2855,14 @@
     </row>
     <row r="20" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W20" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,3)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,3)</f>
         <v>0</v>
       </c>
       <c r="X20" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,3)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,3)</f>
         <v>0</v>
       </c>
       <c r="Y20" s="6">
@@ -2841,14 +2872,14 @@
     </row>
     <row r="21" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W21" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,4)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,4)</f>
         <v>0</v>
       </c>
       <c r="X21" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,4)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,4)</f>
         <v>0</v>
       </c>
       <c r="Y21" s="6">
@@ -2858,14 +2889,14 @@
     </row>
     <row r="22" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="W22" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,5)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,5)</f>
         <v>0</v>
       </c>
       <c r="X22" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,5)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,5)</f>
         <v>0</v>
       </c>
       <c r="Y22" s="6">
@@ -2875,14 +2906,14 @@
     </row>
     <row r="23" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W23" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,6)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,6)</f>
         <v>0</v>
       </c>
       <c r="X23" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,6)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,6)</f>
         <v>0</v>
       </c>
       <c r="Y23" s="6">
@@ -2892,14 +2923,14 @@
     </row>
     <row r="24" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W24" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,7)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,7)</f>
         <v>0</v>
       </c>
       <c r="X24" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,7)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,7)</f>
         <v>0</v>
       </c>
       <c r="Y24" s="6">
@@ -2909,14 +2940,14 @@
     </row>
     <row r="25" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W25" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,8)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,8)</f>
         <v>0</v>
       </c>
       <c r="X25" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,8)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,8)</f>
         <v>0</v>
       </c>
       <c r="Y25" s="6">
@@ -2926,14 +2957,14 @@
     </row>
     <row r="26" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W26" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,9)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,9)</f>
         <v>0</v>
       </c>
       <c r="X26" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,9)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,9)</f>
         <v>0</v>
       </c>
       <c r="Y26" s="6">
@@ -2943,14 +2974,14 @@
     </row>
     <row r="27" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W27" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,10)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,10)</f>
         <v>0</v>
       </c>
       <c r="X27" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,10)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,10)</f>
         <v>0</v>
       </c>
       <c r="Y27" s="6">
@@ -2960,14 +2991,14 @@
     </row>
     <row r="28" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W28" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,11)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,11)</f>
         <v>0</v>
       </c>
       <c r="X28" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,11)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,11)</f>
         <v>0</v>
       </c>
       <c r="Y28" s="6">
@@ -2977,14 +3008,14 @@
     </row>
     <row r="29" spans="22:25" x14ac:dyDescent="0.35">
       <c r="V29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W29" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,12)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,12)</f>
         <v>0</v>
       </c>
       <c r="X29" s="6">
-        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,12)</f>
+        <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,"&lt;&gt;",Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,'Schedule E Summary'!$C$3,Transactions!$H$5:$H$1004,12)</f>
         <v>0</v>
       </c>
       <c r="Y29" s="6">
@@ -2992,15 +3023,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="22:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="W33" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="34" spans="22:23" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+      <c r="X33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V34" t="str">
         <f>'Schedule E Summary'!B8</f>
         <v>Advertising</v>
@@ -3009,8 +3043,12 @@
         <f>'Schedule E Summary'!M8</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X34">
+        <f>W34+100/1000000</f>
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="35" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V35" t="str">
         <f>'Schedule E Summary'!B9</f>
         <v>Auto and travel</v>
@@ -3019,8 +3057,12 @@
         <f>'Schedule E Summary'!M9</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X35">
+        <f>W35+99/1000000</f>
+        <v>9.8999999999999994E-5</v>
+      </c>
+    </row>
+    <row r="36" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V36" t="str">
         <f>'Schedule E Summary'!B10</f>
         <v>Cleaning and maintenance</v>
@@ -3029,8 +3071,12 @@
         <f>'Schedule E Summary'!M10</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X36">
+        <f>W36+98/1000000</f>
+        <v>9.7999999999999997E-5</v>
+      </c>
+    </row>
+    <row r="37" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V37" t="str">
         <f>'Schedule E Summary'!B11</f>
         <v>Commissions</v>
@@ -3039,8 +3085,12 @@
         <f>'Schedule E Summary'!M11</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X37">
+        <f>W37+97/1000000</f>
+        <v>9.7E-5</v>
+      </c>
+    </row>
+    <row r="38" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V38" t="str">
         <f>'Schedule E Summary'!B12</f>
         <v>Insurance</v>
@@ -3049,8 +3099,12 @@
         <f>'Schedule E Summary'!M12</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X38">
+        <f>W38+96/1000000</f>
+        <v>9.6000000000000002E-5</v>
+      </c>
+    </row>
+    <row r="39" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V39" t="str">
         <f>'Schedule E Summary'!B13</f>
         <v>Legal and other professional fees</v>
@@ -3059,8 +3113,12 @@
         <f>'Schedule E Summary'!M13</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X39">
+        <f>W39+95/1000000</f>
+        <v>9.5000000000000005E-5</v>
+      </c>
+    </row>
+    <row r="40" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V40" t="str">
         <f>'Schedule E Summary'!B14</f>
         <v>Management fees</v>
@@ -3069,8 +3127,12 @@
         <f>'Schedule E Summary'!M14</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X40">
+        <f>W40+94/1000000</f>
+        <v>9.3999999999999994E-5</v>
+      </c>
+    </row>
+    <row r="41" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V41" t="str">
         <f>'Schedule E Summary'!B15</f>
         <v>Mortgage interest paid to banks</v>
@@ -3079,8 +3141,12 @@
         <f>'Schedule E Summary'!M15</f>
         <v>612.4</v>
       </c>
-    </row>
-    <row r="42" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X41">
+        <f>W41+93/1000000</f>
+        <v>612.40009299999997</v>
+      </c>
+    </row>
+    <row r="42" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V42" t="str">
         <f>'Schedule E Summary'!B16</f>
         <v>Other interest</v>
@@ -3089,8 +3155,12 @@
         <f>'Schedule E Summary'!M16</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X42">
+        <f>W42+92/1000000</f>
+        <v>9.2E-5</v>
+      </c>
+    </row>
+    <row r="43" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V43" t="str">
         <f>'Schedule E Summary'!B17</f>
         <v>Repairs</v>
@@ -3099,8 +3169,12 @@
         <f>'Schedule E Summary'!M17</f>
         <v>215</v>
       </c>
-    </row>
-    <row r="44" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X43">
+        <f>W43+91/1000000</f>
+        <v>215.000091</v>
+      </c>
+    </row>
+    <row r="44" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V44" t="str">
         <f>'Schedule E Summary'!B18</f>
         <v>Supplies</v>
@@ -3109,8 +3183,12 @@
         <f>'Schedule E Summary'!M18</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X44">
+        <f>W44+90/1000000</f>
+        <v>9.0000000000000006E-5</v>
+      </c>
+    </row>
+    <row r="45" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V45" t="str">
         <f>'Schedule E Summary'!B19</f>
         <v>Taxes</v>
@@ -3119,8 +3197,12 @@
         <f>'Schedule E Summary'!M19</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X45">
+        <f>W45+89/1000000</f>
+        <v>8.8999999999999995E-5</v>
+      </c>
+    </row>
+    <row r="46" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V46" t="str">
         <f>'Schedule E Summary'!B20</f>
         <v>Utilities</v>
@@ -3129,8 +3211,12 @@
         <f>'Schedule E Summary'!M20</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X46">
+        <f>W46+88/1000000</f>
+        <v>8.7999999999999998E-5</v>
+      </c>
+    </row>
+    <row r="47" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V47" t="str">
         <f>'Schedule E Summary'!B21</f>
         <v>Other</v>
@@ -3139,8 +3225,12 @@
         <f>'Schedule E Summary'!M21</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="X47">
+        <f>W47+87/1000000</f>
+        <v>8.7000000000000001E-5</v>
+      </c>
+    </row>
+    <row r="48" spans="22:24" x14ac:dyDescent="0.35">
       <c r="V48" t="str">
         <f>'Schedule E Summary'!B22</f>
         <v>Depreciation (estimated)</v>
@@ -3148,6 +3238,206 @@
       <c r="W48" s="6">
         <f>'Schedule E Summary'!M22</f>
         <v>8181.818181818182</v>
+      </c>
+      <c r="X48">
+        <f>W48+86/1000000</f>
+        <v>8181.818267818182</v>
+      </c>
+    </row>
+    <row r="52" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V52" t="s">
+        <v>48</v>
+      </c>
+      <c r="W52" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="53" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V53" t="str">
+        <f>IF(LARGE($X$34:$X$48,1)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,1),$X$34:$X$48,0)))</f>
+        <v>Depreciation (estimated)</v>
+      </c>
+      <c r="W53" s="6">
+        <f>IF(LARGE($X$34:$X$48,1)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,1),2))</f>
+        <v>8181.82</v>
+      </c>
+    </row>
+    <row r="54" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V54" t="str">
+        <f>IF(LARGE($X$34:$X$48,2)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,2),$X$34:$X$48,0)))</f>
+        <v>Mortgage interest paid to banks</v>
+      </c>
+      <c r="W54" s="6">
+        <f>IF(LARGE($X$34:$X$48,2)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,2),2))</f>
+        <v>612.4</v>
+      </c>
+    </row>
+    <row r="55" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V55" t="str">
+        <f>IF(LARGE($X$34:$X$48,3)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,3),$X$34:$X$48,0)))</f>
+        <v>Repairs</v>
+      </c>
+      <c r="W55" s="6">
+        <f>IF(LARGE($X$34:$X$48,3)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,3),2))</f>
+        <v>215</v>
+      </c>
+    </row>
+    <row r="56" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V56" t="str">
+        <f>IF(LARGE($X$34:$X$48,4)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,4),$X$34:$X$48,0)))</f>
+        <v/>
+      </c>
+      <c r="W56" s="6">
+        <f>IF(LARGE($X$34:$X$48,4)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,4),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V57" t="str">
+        <f>IF(LARGE($X$34:$X$48,5)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,5),$X$34:$X$48,0)))</f>
+        <v/>
+      </c>
+      <c r="W57" s="6">
+        <f>IF(LARGE($X$34:$X$48,5)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,5),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V58" t="str">
+        <f>IF(LARGE($X$34:$X$48,6)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,6),$X$34:$X$48,0)))</f>
+        <v/>
+      </c>
+      <c r="W58" s="6">
+        <f>IF(LARGE($X$34:$X$48,6)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,6),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V59" t="str">
+        <f>IF(LARGE($X$34:$X$48,7)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,7),$X$34:$X$48,0)))</f>
+        <v/>
+      </c>
+      <c r="W59" s="6">
+        <f>IF(LARGE($X$34:$X$48,7)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,7),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V60" t="str">
+        <f>IF(LARGE($X$34:$X$48,8)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,8),$X$34:$X$48,0)))</f>
+        <v/>
+      </c>
+      <c r="W60" s="6">
+        <f>IF(LARGE($X$34:$X$48,8)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,8),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V62" t="s">
+        <v>49</v>
+      </c>
+      <c r="W62" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V63" t="str">
+        <f>IF(LARGE($X$5:$X$14,1)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,1),$X$5:$X$14,0)))</f>
+        <v>EXAMPLE: 412 Maple St (duplex)</v>
+      </c>
+      <c r="W63" s="6">
+        <f>IF(LARGE($X$5:$X$14,1)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,1),2))</f>
+        <v>-7559.22</v>
+      </c>
+    </row>
+    <row r="64" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V64" t="str">
+        <f>IF(LARGE($X$5:$X$14,2)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,2),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W64" s="6">
+        <f>IF(LARGE($X$5:$X$14,2)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,2),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V65" t="str">
+        <f>IF(LARGE($X$5:$X$14,3)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,3),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W65" s="6">
+        <f>IF(LARGE($X$5:$X$14,3)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,3),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V66" t="str">
+        <f>IF(LARGE($X$5:$X$14,4)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,4),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W66" s="6">
+        <f>IF(LARGE($X$5:$X$14,4)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,4),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V67" t="str">
+        <f>IF(LARGE($X$5:$X$14,5)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,5),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W67" s="6">
+        <f>IF(LARGE($X$5:$X$14,5)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,5),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V68" t="str">
+        <f>IF(LARGE($X$5:$X$14,6)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,6),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W68" s="6">
+        <f>IF(LARGE($X$5:$X$14,6)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,6),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V69" t="str">
+        <f>IF(LARGE($X$5:$X$14,7)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,7),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W69" s="6">
+        <f>IF(LARGE($X$5:$X$14,7)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,7),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V70" t="str">
+        <f>IF(LARGE($X$5:$X$14,8)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,8),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W70" s="6">
+        <f>IF(LARGE($X$5:$X$14,8)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,8),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V71" t="str">
+        <f>IF(LARGE($X$5:$X$14,9)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,9),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W71" s="6">
+        <f>IF(LARGE($X$5:$X$14,9)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,9),2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="22:23" x14ac:dyDescent="0.35">
+      <c r="V72" t="str">
+        <f>IF(LARGE($X$5:$X$14,10)&lt;-100000000000,"",INDEX($V$5:$V$14,MATCH(LARGE($X$5:$X$14,10),$X$5:$X$14,0)))</f>
+        <v/>
+      </c>
+      <c r="W72" s="6">
+        <f>IF(LARGE($X$5:$X$14,10)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,10),2))</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3190,41 +3480,41 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -3232,7 +3522,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C5" s="9">
         <v>2</v>
@@ -3459,7 +3749,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -3486,38 +3776,41 @@
   <sheetData>
     <row r="1" spans="1:8" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>24</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -3525,13 +3818,13 @@
         <v>46023</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E5" s="11">
         <v>1450</v>
@@ -3554,13 +3847,13 @@
         <v>46031</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E6" s="11">
         <v>215</v>
@@ -3583,13 +3876,13 @@
         <v>46053</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E7" s="11">
         <v>612.4</v>
@@ -22551,6 +22844,21 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A5:A1004">
+    <cfRule type="expression" dxfId="4" priority="3">
+      <formula>AND(A5="",E5&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:B1004">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>AND(B5="",OR(A5&lt;&gt;"",E5&lt;&gt;""))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:C1004">
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>OR(F5="?",AND(C5="",E5&lt;&gt;""))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -22589,26 +22897,26 @@
   <sheetData>
     <row r="1" spans="1:13" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="14">
+      <c r="B3" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="15">
         <v>2026</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C5" s="7" t="str">
         <f>IF(Properties!B5="","Property 1",Properties!B5)</f>
@@ -22651,1052 +22959,1052 @@
         <v>Property 10</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="16">
+      <c r="A6" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>1450</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I6" s="16">
+      <c r="I6" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J6" s="16">
+      <c r="J6" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K6" s="16">
+      <c r="K6" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L6" s="16">
+      <c r="L6" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B6,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M6" s="17">
+      <c r="M6" s="18">
         <f t="shared" ref="M6:M22" si="0">SUM(C6:L6)</f>
         <v>1450</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="18">
+        <v>83</v>
+      </c>
+      <c r="C7" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I7" s="18">
+      <c r="I7" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J7" s="18">
+      <c r="J7" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B7,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M7" s="19">
+      <c r="M7" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="16">
+      <c r="A8" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H8" s="16">
+      <c r="H8" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I8" s="16">
+      <c r="I8" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J8" s="16">
+      <c r="J8" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K8" s="16">
+      <c r="K8" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L8" s="16">
+      <c r="L8" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B8,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M8" s="17">
+      <c r="M8" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C9" s="18">
+        <v>87</v>
+      </c>
+      <c r="C9" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J9" s="18">
+      <c r="J9" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K9" s="18">
+      <c r="K9" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L9" s="18">
+      <c r="L9" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B9,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M9" s="19">
+      <c r="M9" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" s="16">
+      <c r="A10" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H10" s="16">
+      <c r="H10" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J10" s="16">
+      <c r="J10" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K10" s="16">
+      <c r="K10" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B10,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M10" s="17">
+      <c r="M10" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="C11" s="18">
+        <v>91</v>
+      </c>
+      <c r="C11" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B11,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M11" s="19">
+      <c r="M11" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="C12" s="16">
+      <c r="A12" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H12" s="16">
+      <c r="H12" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J12" s="16">
+      <c r="J12" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K12" s="16">
+      <c r="K12" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L12" s="16">
+      <c r="L12" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B12,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M12" s="17">
+      <c r="M12" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C13" s="18">
+        <v>95</v>
+      </c>
+      <c r="C13" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J13" s="18">
+      <c r="J13" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K13" s="18">
+      <c r="K13" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L13" s="18">
+      <c r="L13" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B13,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M13" s="19">
+      <c r="M13" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="16">
+      <c r="A14" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H14" s="16">
+      <c r="H14" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J14" s="16">
+      <c r="J14" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K14" s="16">
+      <c r="K14" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L14" s="16">
+      <c r="L14" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B14,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M14" s="17">
+      <c r="M14" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="18">
+        <v>75</v>
+      </c>
+      <c r="C15" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>612.4</v>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J15" s="18">
+      <c r="J15" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K15" s="18">
+      <c r="K15" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L15" s="18">
+      <c r="L15" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B15,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M15" s="19">
+      <c r="M15" s="20">
         <f t="shared" si="0"/>
         <v>612.4</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="C16" s="16">
+      <c r="A16" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H16" s="16">
+      <c r="H16" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B16,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M16" s="17">
+      <c r="M16" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C17" s="18">
+        <v>73</v>
+      </c>
+      <c r="C17" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>215</v>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J17" s="18">
+      <c r="J17" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K17" s="18">
+      <c r="K17" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L17" s="18">
+      <c r="L17" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B17,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M17" s="19">
+      <c r="M17" s="20">
         <f t="shared" si="0"/>
         <v>215</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A18" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C18" s="16">
+      <c r="A18" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H18" s="16">
+      <c r="H18" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J18" s="16">
+      <c r="J18" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K18" s="16">
+      <c r="K18" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L18" s="16">
+      <c r="L18" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B18,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M18" s="17">
+      <c r="M18" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="C19" s="18">
+        <v>105</v>
+      </c>
+      <c r="C19" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L19" s="18">
+      <c r="L19" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B19,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M19" s="19">
+      <c r="M19" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A20" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>103</v>
-      </c>
-      <c r="C20" s="16">
+      <c r="A20" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D20" s="16">
+      <c r="D20" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="17">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="17">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="17">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H20" s="16">
+      <c r="H20" s="17">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="17">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="17">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K20" s="16">
+      <c r="K20" s="17">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L20" s="16">
+      <c r="L20" s="17">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B20,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M20" s="17">
+      <c r="M20" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="C21" s="18">
+        <v>109</v>
+      </c>
+      <c r="C21" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="19">
         <f>IF(Properties!$B$7="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$7,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="19">
         <f>IF(Properties!$B$8="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$8,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="19">
         <f>IF(Properties!$B$9="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$9,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="19">
         <f>IF(Properties!$B$10="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$10,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="19">
         <f>IF(Properties!$B$11="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$11,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="J21" s="18">
+      <c r="J21" s="19">
         <f>IF(Properties!$B$12="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$12,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="K21" s="18">
+      <c r="K21" s="19">
         <f>IF(Properties!$B$13="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$13,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="L21" s="18">
+      <c r="L21" s="19">
         <f>IF(Properties!$B$14="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$14,Transactions!$C$5:$C$1004,$B21,Transactions!$G$5:$G$1004,$C$3))</f>
         <v>0</v>
       </c>
-      <c r="M21" s="19">
+      <c r="M21" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C22" s="20">
+        <v>111</v>
+      </c>
+      <c r="C22" s="21">
         <f>Properties!I5</f>
         <v>8181.818181818182</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="21">
         <f>Properties!I6</f>
         <v>0</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="21">
         <f>Properties!I7</f>
         <v>0</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="21">
         <f>Properties!I8</f>
         <v>0</v>
       </c>
-      <c r="G22" s="20">
+      <c r="G22" s="21">
         <f>Properties!I9</f>
         <v>0</v>
       </c>
-      <c r="H22" s="20">
+      <c r="H22" s="21">
         <f>Properties!I10</f>
         <v>0</v>
       </c>
-      <c r="I22" s="20">
+      <c r="I22" s="21">
         <f>Properties!I11</f>
         <v>0</v>
       </c>
-      <c r="J22" s="20">
+      <c r="J22" s="21">
         <f>Properties!I12</f>
         <v>0</v>
       </c>
-      <c r="K22" s="20">
+      <c r="K22" s="21">
         <f>Properties!I13</f>
         <v>0</v>
       </c>
-      <c r="L22" s="20">
+      <c r="L22" s="21">
         <f>Properties!I14</f>
         <v>0</v>
       </c>
-      <c r="M22" s="19">
+      <c r="M22" s="20">
         <f t="shared" si="0"/>
         <v>8181.818181818182</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B24" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="C24" s="19">
+      <c r="B24" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" s="20">
         <f t="shared" ref="C24:M24" si="1">C6+C7</f>
         <v>1450</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I24" s="19">
+      <c r="I24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J24" s="19">
+      <c r="J24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K24" s="19">
+      <c r="K24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L24" s="19">
+      <c r="L24" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="M24" s="19">
+      <c r="M24" s="20">
         <f t="shared" si="1"/>
         <v>1450</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B25" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C25" s="19">
+      <c r="B25" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C25" s="20">
         <f t="shared" ref="C25:M25" si="2">C8+C9+C10+C11+C12+C13+C14+C15+C16+C17+C18+C19+C20+C21+C22</f>
         <v>9009.2181818181816</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I25" s="19">
+      <c r="I25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J25" s="19">
+      <c r="J25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K25" s="19">
+      <c r="K25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L25" s="19">
+      <c r="L25" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M25" s="19">
+      <c r="M25" s="20">
         <f t="shared" si="2"/>
         <v>9009.2181818181816</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B26" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="C26" s="22">
+      <c r="B26" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="23">
         <f t="shared" ref="C26:M26" si="3">C24-C25</f>
         <v>-7559.2181818181816</v>
       </c>
-      <c r="D26" s="22">
+      <c r="D26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F26" s="22">
+      <c r="F26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H26" s="22">
+      <c r="H26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I26" s="22">
+      <c r="I26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J26" s="22">
+      <c r="J26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K26" s="22">
+      <c r="K26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L26" s="22">
+      <c r="L26" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M26" s="22">
+      <c r="M26" s="23">
         <f t="shared" si="3"/>
         <v>-7559.2181818181816</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B28" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C28" s="23">
+        <v>115</v>
+      </c>
+      <c r="C28" s="24">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$G$5:$G$1004,$C$3)-SUM(M6:M21)</f>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B29" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -23720,46 +24028,46 @@
   <sheetData>
     <row r="1" spans="1:6" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B3" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>115</v>
+      <c r="B3" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B4" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="25">
+      <c r="B4" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="26">
         <f>'Schedule E Summary'!C3</f>
         <v>2026</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B6" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B7" s="26" t="s">
-        <v>33</v>
+      <c r="B7" s="27" t="s">
+        <v>34</v>
       </c>
       <c r="C7" s="12">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,1)</f>
@@ -23779,29 +24087,29 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B8" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="28">
+      <c r="B8" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,2)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,2)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="28">
+      <c r="E8" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="28">
+      <c r="F8" s="29">
         <f>SUM($E$7:E8)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="26" t="s">
-        <v>35</v>
+      <c r="B9" s="27" t="s">
+        <v>36</v>
       </c>
       <c r="C9" s="12">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,3)</f>
@@ -23821,29 +24129,29 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="28">
+      <c r="B10" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,4)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,4)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="29">
         <f>SUM($E$7:E10)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="26" t="s">
-        <v>37</v>
+      <c r="B11" s="27" t="s">
+        <v>38</v>
       </c>
       <c r="C11" s="12">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,5)</f>
@@ -23863,29 +24171,29 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B12" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="28">
+      <c r="B12" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,6)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,6)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F12" s="28">
+      <c r="F12" s="29">
         <f>SUM($E$7:E12)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="26" t="s">
-        <v>39</v>
+      <c r="B13" s="27" t="s">
+        <v>40</v>
       </c>
       <c r="C13" s="12">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,7)</f>
@@ -23905,29 +24213,29 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="28">
+      <c r="B14" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,8)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,8)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="28">
+      <c r="E14" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F14" s="28">
+      <c r="F14" s="29">
         <f>SUM($E$7:E14)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B15" s="26" t="s">
-        <v>41</v>
+      <c r="B15" s="27" t="s">
+        <v>42</v>
       </c>
       <c r="C15" s="12">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,9)</f>
@@ -23947,29 +24255,29 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B16" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="28">
+      <c r="B16" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,10)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,10)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="28">
+      <c r="E16" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F16" s="28">
+      <c r="F16" s="29">
         <f>SUM($E$7:E16)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B17" s="26" t="s">
-        <v>43</v>
+      <c r="B17" s="27" t="s">
+        <v>44</v>
       </c>
       <c r="C17" s="12">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,11)</f>
@@ -23989,46 +24297,46 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B18" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="28">
+      <c r="B18" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Income",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,12)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="29">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,IF($C$3="All properties","*",$C$3),Transactions!$F$5:$F$1004,"Expense",Transactions!$G$5:$G$1004,$C$4,Transactions!$H$5:$H$1004,12)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="28">
+      <c r="E18" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="28">
+      <c r="F18" s="29">
         <f>SUM($E$7:E18)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B19" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="C19" s="19">
+      <c r="B19" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="20">
         <f>SUM(C7:C18)</f>
         <v>1450</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="20">
         <f>SUM(D7:D18)</f>
         <v>827.4</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="20">
         <f>SUM(E7:E18)</f>
         <v>622.6</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -24068,12 +24376,12 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -24081,42 +24389,42 @@
         <v>24</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E5" s="11">
         <v>1450</v>
@@ -24130,7 +24438,7 @@
       <c r="H5" s="10">
         <v>46599</v>
       </c>
-      <c r="I5" s="26">
+      <c r="I5" s="27">
         <f t="shared" ref="I5:I36" ca="1" si="0">IF(H5="","",H5-TODAY())</f>
         <v>282</v>
       </c>
@@ -24144,7 +24452,7 @@
       <c r="F6" s="11"/>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
-      <c r="I6" s="26" t="str">
+      <c r="I6" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24158,7 +24466,7 @@
       <c r="F7" s="11"/>
       <c r="G7" s="10"/>
       <c r="H7" s="10"/>
-      <c r="I7" s="26" t="str">
+      <c r="I7" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24172,7 +24480,7 @@
       <c r="F8" s="11"/>
       <c r="G8" s="10"/>
       <c r="H8" s="10"/>
-      <c r="I8" s="26" t="str">
+      <c r="I8" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24186,7 +24494,7 @@
       <c r="F9" s="11"/>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
-      <c r="I9" s="26" t="str">
+      <c r="I9" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24200,7 +24508,7 @@
       <c r="F10" s="11"/>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
-      <c r="I10" s="26" t="str">
+      <c r="I10" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24214,7 +24522,7 @@
       <c r="F11" s="11"/>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
-      <c r="I11" s="26" t="str">
+      <c r="I11" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24228,7 +24536,7 @@
       <c r="F12" s="11"/>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
-      <c r="I12" s="26" t="str">
+      <c r="I12" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24242,7 +24550,7 @@
       <c r="F13" s="11"/>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
-      <c r="I13" s="26" t="str">
+      <c r="I13" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24256,7 +24564,7 @@
       <c r="F14" s="11"/>
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
-      <c r="I14" s="26" t="str">
+      <c r="I14" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24270,7 +24578,7 @@
       <c r="F15" s="11"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="26" t="str">
+      <c r="I15" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24284,7 +24592,7 @@
       <c r="F16" s="11"/>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
-      <c r="I16" s="26" t="str">
+      <c r="I16" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24298,7 +24606,7 @@
       <c r="F17" s="11"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
-      <c r="I17" s="26" t="str">
+      <c r="I17" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24312,7 +24620,7 @@
       <c r="F18" s="11"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
-      <c r="I18" s="26" t="str">
+      <c r="I18" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24326,7 +24634,7 @@
       <c r="F19" s="11"/>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
-      <c r="I19" s="26" t="str">
+      <c r="I19" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24340,7 +24648,7 @@
       <c r="F20" s="11"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
-      <c r="I20" s="26" t="str">
+      <c r="I20" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24354,7 +24662,7 @@
       <c r="F21" s="11"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
-      <c r="I21" s="26" t="str">
+      <c r="I21" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24368,7 +24676,7 @@
       <c r="F22" s="11"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
-      <c r="I22" s="26" t="str">
+      <c r="I22" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24382,7 +24690,7 @@
       <c r="F23" s="11"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
-      <c r="I23" s="26" t="str">
+      <c r="I23" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24396,7 +24704,7 @@
       <c r="F24" s="11"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
-      <c r="I24" s="26" t="str">
+      <c r="I24" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24410,7 +24718,7 @@
       <c r="F25" s="11"/>
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
-      <c r="I25" s="26" t="str">
+      <c r="I25" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24424,7 +24732,7 @@
       <c r="F26" s="11"/>
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
-      <c r="I26" s="26" t="str">
+      <c r="I26" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24438,7 +24746,7 @@
       <c r="F27" s="11"/>
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
-      <c r="I27" s="26" t="str">
+      <c r="I27" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24452,7 +24760,7 @@
       <c r="F28" s="11"/>
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
-      <c r="I28" s="26" t="str">
+      <c r="I28" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24466,7 +24774,7 @@
       <c r="F29" s="11"/>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
-      <c r="I29" s="26" t="str">
+      <c r="I29" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24480,7 +24788,7 @@
       <c r="F30" s="11"/>
       <c r="G30" s="10"/>
       <c r="H30" s="10"/>
-      <c r="I30" s="26" t="str">
+      <c r="I30" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24494,7 +24802,7 @@
       <c r="F31" s="11"/>
       <c r="G31" s="10"/>
       <c r="H31" s="10"/>
-      <c r="I31" s="26" t="str">
+      <c r="I31" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24508,7 +24816,7 @@
       <c r="F32" s="11"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
-      <c r="I32" s="26" t="str">
+      <c r="I32" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24522,7 +24830,7 @@
       <c r="F33" s="11"/>
       <c r="G33" s="10"/>
       <c r="H33" s="10"/>
-      <c r="I33" s="26" t="str">
+      <c r="I33" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24536,7 +24844,7 @@
       <c r="F34" s="11"/>
       <c r="G34" s="10"/>
       <c r="H34" s="10"/>
-      <c r="I34" s="26" t="str">
+      <c r="I34" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24550,7 +24858,7 @@
       <c r="F35" s="11"/>
       <c r="G35" s="10"/>
       <c r="H35" s="10"/>
-      <c r="I35" s="26" t="str">
+      <c r="I35" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24564,7 +24872,7 @@
       <c r="F36" s="11"/>
       <c r="G36" s="10"/>
       <c r="H36" s="10"/>
-      <c r="I36" s="26" t="str">
+      <c r="I36" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
         <v/>
       </c>
@@ -24578,7 +24886,7 @@
       <c r="F37" s="11"/>
       <c r="G37" s="10"/>
       <c r="H37" s="10"/>
-      <c r="I37" s="26" t="str">
+      <c r="I37" s="27" t="str">
         <f t="shared" ref="I37:I68" ca="1" si="1">IF(H37="","",H37-TODAY())</f>
         <v/>
       </c>
@@ -24592,7 +24900,7 @@
       <c r="F38" s="11"/>
       <c r="G38" s="10"/>
       <c r="H38" s="10"/>
-      <c r="I38" s="26" t="str">
+      <c r="I38" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24606,7 +24914,7 @@
       <c r="F39" s="11"/>
       <c r="G39" s="10"/>
       <c r="H39" s="10"/>
-      <c r="I39" s="26" t="str">
+      <c r="I39" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24620,7 +24928,7 @@
       <c r="F40" s="11"/>
       <c r="G40" s="10"/>
       <c r="H40" s="10"/>
-      <c r="I40" s="26" t="str">
+      <c r="I40" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24634,7 +24942,7 @@
       <c r="F41" s="11"/>
       <c r="G41" s="10"/>
       <c r="H41" s="10"/>
-      <c r="I41" s="26" t="str">
+      <c r="I41" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24648,7 +24956,7 @@
       <c r="F42" s="11"/>
       <c r="G42" s="10"/>
       <c r="H42" s="10"/>
-      <c r="I42" s="26" t="str">
+      <c r="I42" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24662,7 +24970,7 @@
       <c r="F43" s="11"/>
       <c r="G43" s="10"/>
       <c r="H43" s="10"/>
-      <c r="I43" s="26" t="str">
+      <c r="I43" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24676,7 +24984,7 @@
       <c r="F44" s="11"/>
       <c r="G44" s="10"/>
       <c r="H44" s="10"/>
-      <c r="I44" s="26" t="str">
+      <c r="I44" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24690,7 +24998,7 @@
       <c r="F45" s="11"/>
       <c r="G45" s="10"/>
       <c r="H45" s="10"/>
-      <c r="I45" s="26" t="str">
+      <c r="I45" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24704,7 +25012,7 @@
       <c r="F46" s="11"/>
       <c r="G46" s="10"/>
       <c r="H46" s="10"/>
-      <c r="I46" s="26" t="str">
+      <c r="I46" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24718,7 +25026,7 @@
       <c r="F47" s="11"/>
       <c r="G47" s="10"/>
       <c r="H47" s="10"/>
-      <c r="I47" s="26" t="str">
+      <c r="I47" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24732,7 +25040,7 @@
       <c r="F48" s="11"/>
       <c r="G48" s="10"/>
       <c r="H48" s="10"/>
-      <c r="I48" s="26" t="str">
+      <c r="I48" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24746,7 +25054,7 @@
       <c r="F49" s="11"/>
       <c r="G49" s="10"/>
       <c r="H49" s="10"/>
-      <c r="I49" s="26" t="str">
+      <c r="I49" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24760,7 +25068,7 @@
       <c r="F50" s="11"/>
       <c r="G50" s="10"/>
       <c r="H50" s="10"/>
-      <c r="I50" s="26" t="str">
+      <c r="I50" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24774,7 +25082,7 @@
       <c r="F51" s="11"/>
       <c r="G51" s="10"/>
       <c r="H51" s="10"/>
-      <c r="I51" s="26" t="str">
+      <c r="I51" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24788,7 +25096,7 @@
       <c r="F52" s="11"/>
       <c r="G52" s="10"/>
       <c r="H52" s="10"/>
-      <c r="I52" s="26" t="str">
+      <c r="I52" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24802,7 +25110,7 @@
       <c r="F53" s="11"/>
       <c r="G53" s="10"/>
       <c r="H53" s="10"/>
-      <c r="I53" s="26" t="str">
+      <c r="I53" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24816,7 +25124,7 @@
       <c r="F54" s="11"/>
       <c r="G54" s="10"/>
       <c r="H54" s="10"/>
-      <c r="I54" s="26" t="str">
+      <c r="I54" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24830,7 +25138,7 @@
       <c r="F55" s="11"/>
       <c r="G55" s="10"/>
       <c r="H55" s="10"/>
-      <c r="I55" s="26" t="str">
+      <c r="I55" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24844,7 +25152,7 @@
       <c r="F56" s="11"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10"/>
-      <c r="I56" s="26" t="str">
+      <c r="I56" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24858,7 +25166,7 @@
       <c r="F57" s="11"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10"/>
-      <c r="I57" s="26" t="str">
+      <c r="I57" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24872,7 +25180,7 @@
       <c r="F58" s="11"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10"/>
-      <c r="I58" s="26" t="str">
+      <c r="I58" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24886,7 +25194,7 @@
       <c r="F59" s="11"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10"/>
-      <c r="I59" s="26" t="str">
+      <c r="I59" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24900,7 +25208,7 @@
       <c r="F60" s="11"/>
       <c r="G60" s="10"/>
       <c r="H60" s="10"/>
-      <c r="I60" s="26" t="str">
+      <c r="I60" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24914,7 +25222,7 @@
       <c r="F61" s="11"/>
       <c r="G61" s="10"/>
       <c r="H61" s="10"/>
-      <c r="I61" s="26" t="str">
+      <c r="I61" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24928,7 +25236,7 @@
       <c r="F62" s="11"/>
       <c r="G62" s="10"/>
       <c r="H62" s="10"/>
-      <c r="I62" s="26" t="str">
+      <c r="I62" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24942,7 +25250,7 @@
       <c r="F63" s="11"/>
       <c r="G63" s="10"/>
       <c r="H63" s="10"/>
-      <c r="I63" s="26" t="str">
+      <c r="I63" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
@@ -24956,16 +25264,16 @@
       <c r="F64" s="11"/>
       <c r="G64" s="10"/>
       <c r="H64" s="10"/>
-      <c r="I64" s="26" t="str">
+      <c r="I64" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
         <v/>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A66" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="E66" s="19">
+      <c r="A66" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="E66" s="20">
         <f>SUM(E5:E64)</f>
         <v>1450</v>
       </c>
@@ -25005,41 +25313,41 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" t="str">
         <f>IF(Properties!B5="","",Properties!B5)</f>
@@ -25048,13 +25356,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E4" t="str">
         <f>IF(Properties!B6="","",Properties!B6)</f>
@@ -25063,13 +25371,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C5" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E5" t="str">
         <f>IF(Properties!B7="","",Properties!B7)</f>
@@ -25078,13 +25386,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E6" t="str">
         <f>IF(Properties!B8="","",Properties!B8)</f>
@@ -25093,13 +25401,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E7" t="str">
         <f>IF(Properties!B9="","",Properties!B9)</f>
@@ -25108,13 +25416,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E8" t="str">
         <f>IF(Properties!B10="","",Properties!B10)</f>
@@ -25123,13 +25431,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E9" t="str">
         <f>IF(Properties!B11="","",Properties!B11)</f>
@@ -25138,13 +25446,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E10" t="str">
         <f>IF(Properties!B12="","",Properties!B12)</f>
@@ -25153,13 +25461,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E11" t="str">
         <f>IF(Properties!B13="","",Properties!B13)</f>
@@ -25168,13 +25476,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E12" t="str">
         <f>IF(Properties!B14="","",Properties!B14)</f>
@@ -25183,57 +25491,57 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B16" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C16" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C17" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Review fixes: rental example year, remove placeholder product cards, accurate delivery copy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dl/QkFNAj8Wx9bU9aQs/Rental-Property-Tracker-NoraStudio.xlsx
+++ b/dl/QkFNAj8Wx9bU9aQs/Rental-Property-Tracker-NoraStudio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\Joker\projects\products\01-rental-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75577D26-FD45-4327-9E62-BC127DD5C693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9725692F-3F32-45E3-9374-593961C04CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34290" yWindow="-210" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="169">
   <si>
     <t>Rental Property Tracker</t>
   </si>
@@ -54,7 +54,7 @@
     <t>1. Set your tax year on the 'Schedule E Summary' tab (cell C3). The 'Dashboard' tab shows your whole portfolio at a glance.</t>
   </si>
   <si>
-    <t>2. 'Properties' tab: enter each property's name, purchase date, price and land value in the yellow cells. Delete the example row first.</t>
+    <t>2. 'Properties' tab: enter each property's name, purchase date, price and land value in the yellow cells. First clear the EXAMPLE rows: Properties row 5, Transactions rows 5-28 and Rent Roll rows 5-6 (select the yellow cells, press Delete).</t>
   </si>
   <si>
     <t>3. 'Transactions' tab: log every rent payment and expense. Pick property and category from the dropdowns; enter amounts as positive numbers.</t>
@@ -264,7 +264,7 @@
     <t>Rents received</t>
   </si>
   <si>
-    <t>Unit A - January rent</t>
+    <t>Units A+B - January rent</t>
   </si>
   <si>
     <t>Repairs</t>
@@ -277,6 +277,75 @@
   </si>
   <si>
     <t>Bank - January interest</t>
+  </si>
+  <si>
+    <t>Units A+B - February rent</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Landlord policy - annual</t>
+  </si>
+  <si>
+    <t>Bank - February interest</t>
+  </si>
+  <si>
+    <t>Units A+B - March rent</t>
+  </si>
+  <si>
+    <t>Bank - March interest</t>
+  </si>
+  <si>
+    <t>Units A+B - April rent</t>
+  </si>
+  <si>
+    <t>Taxes</t>
+  </si>
+  <si>
+    <t>Property tax - 1st half</t>
+  </si>
+  <si>
+    <t>Bank - April interest</t>
+  </si>
+  <si>
+    <t>Units A+B - May rent</t>
+  </si>
+  <si>
+    <t>Bank - May interest</t>
+  </si>
+  <si>
+    <t>Units A+B - June rent</t>
+  </si>
+  <si>
+    <t>Bank - June interest</t>
+  </si>
+  <si>
+    <t>Units A+B - July rent</t>
+  </si>
+  <si>
+    <t>Bank - July interest</t>
+  </si>
+  <si>
+    <t>Units A+B - August rent</t>
+  </si>
+  <si>
+    <t>Bank - August interest</t>
+  </si>
+  <si>
+    <t>Units A+B - September rent</t>
+  </si>
+  <si>
+    <t>Bank - September interest</t>
+  </si>
+  <si>
+    <t>Units A+B - October rent</t>
+  </si>
+  <si>
+    <t>Property tax - 2nd half</t>
+  </si>
+  <si>
+    <t>Bank - October interest</t>
   </si>
   <si>
     <t>Schedule E Summary</t>
@@ -327,9 +396,6 @@
     <t>9</t>
   </si>
   <si>
-    <t>Insurance</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
@@ -361,9 +427,6 @@
   </si>
   <si>
     <t>16</t>
-  </si>
-  <si>
-    <t>Taxes</t>
   </si>
   <si>
     <t>17</t>
@@ -457,6 +520,15 @@
   </si>
   <si>
     <t>jrivera@email.com</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>M. Chen</t>
+  </si>
+  <si>
+    <t>mchen@email.com</t>
   </si>
   <si>
     <t>Total monthly rent:</t>
@@ -872,34 +944,34 @@
                 <c:formatCode>\$#,##0.00;\(\$#,##0.00\);"-"</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>1450</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -912,7 +984,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9094-42B3-A371-26EF2721CB4F}"/>
+              <c16:uniqueId val="{00000000-CFEA-4A5A-B5F0-5FDF4F0F7B00}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -996,31 +1068,31 @@
                   <c:v>827.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1662.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>2037.4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>2037.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -1033,7 +1105,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9094-42B3-A371-26EF2721CB4F}"/>
+              <c16:uniqueId val="{00000001-CFEA-4A5A-B5F0-5FDF4F0F7B00}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1161,7 +1233,7 @@
             <c:strRef>
               <c:f>Dashboard!$V$53:$V$60</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>Depreciation (estimated)</c:v>
                 </c:pt>
@@ -1169,6 +1241,12 @@
                   <c:v>Mortgage interest paid to banks</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>Taxes</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Insurance</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Repairs</c:v>
                 </c:pt>
               </c:strCache>
@@ -1184,16 +1262,16 @@
                   <c:v>8181.82</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>612.4</c:v>
+                  <c:v>6124</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>215</c:v>
+                  <c:v>2850</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1050</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>215</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1209,7 +1287,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FFDB-4ACE-9851-7D7C83B9C7F6}"/>
+              <c16:uniqueId val="{00000000-73C6-43F4-A7C2-D9816F7BB9AB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1347,7 +1425,7 @@
                 <c:formatCode>\$#,##0.00;\(\$#,##0.00\);"-"</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>-7559.22</c:v>
+                  <c:v>10029.18</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1381,7 +1459,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-CB56-42A1-8AF6-8E29B78A3921}"/>
+              <c16:uniqueId val="{00000000-E796-4DD7-94E8-F06A6A412489}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1552,34 +1630,34 @@
                 <c:formatCode>\$#,##0.00;\(\$#,##0.00\);"-"</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>622.6</c:v>
+                  <c:v>2017.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1182.5999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2232.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>807.59999999999991</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2232.6</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>2232.6</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>2232.6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>2232.6</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>2232.6</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>807.59999999999991</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -1592,7 +1670,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C848-444D-97DC-8B2D2C69AB23}"/>
+              <c16:uniqueId val="{00000000-512E-427F-8185-AC32D7BBB241}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1763,34 +1841,34 @@
                 <c:formatCode>\$#,##0.00;\(\$#,##0.00\);"-"</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>1450</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>2845</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -1818,7 +1896,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0ACF-4F8B-A546-F056DEA4C7A0}"/>
+              <c16:uniqueId val="{00000000-7345-4423-AE73-69832CC07187}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1902,31 +1980,31 @@
                   <c:v>827.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1662.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>2037.4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>612.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>2037.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -1954,7 +2032,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0ACF-4F8B-A546-F056DEA4C7A0}"/>
+              <c16:uniqueId val="{00000001-7345-4423-AE73-69832CC07187}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2667,21 +2745,21 @@
     <row r="5" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B5" s="30">
         <f>'Schedule E Summary'!M24</f>
-        <v>1450</v>
+        <v>28450</v>
       </c>
       <c r="C5" s="31"/>
       <c r="D5" s="31"/>
       <c r="E5" s="31"/>
       <c r="G5" s="30">
         <f>'Schedule E Summary'!M25</f>
-        <v>9009.2181818181816</v>
+        <v>18420.818181818184</v>
       </c>
       <c r="H5" s="31"/>
       <c r="I5" s="31"/>
       <c r="J5" s="31"/>
       <c r="L5" s="30">
         <f>'Schedule E Summary'!M26</f>
-        <v>-7559.2181818181816</v>
+        <v>10029.181818181816</v>
       </c>
       <c r="M5" s="31"/>
       <c r="N5" s="31"/>
@@ -2692,11 +2770,11 @@
       </c>
       <c r="W5" s="6">
         <f>IF(Properties!B5="",0,'Schedule E Summary'!C26)</f>
-        <v>-7559.2181818181816</v>
+        <v>10029.181818181816</v>
       </c>
       <c r="X5">
         <f>IF(V5="",-1000000000000,W5)+20/1000000</f>
-        <v>-7559.2181618181812</v>
+        <v>10029.181838181816</v>
       </c>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.35">
@@ -2774,14 +2852,14 @@
     <row r="9" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B9" s="30">
         <f>'Schedule E Summary'!M24-('Schedule E Summary'!M25-'Schedule E Summary'!M22)</f>
-        <v>622.60000000000036</v>
+        <v>18211</v>
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="31"/>
       <c r="E9" s="31"/>
       <c r="G9" s="30">
         <f>'Rent Roll'!E66</f>
-        <v>1450</v>
+        <v>2845</v>
       </c>
       <c r="H9" s="31"/>
       <c r="I9" s="31"/>
@@ -2908,7 +2986,7 @@
       </c>
       <c r="W18" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,1,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,2,1)),Transactions!$E$5:$E$1004)</f>
-        <v>1450</v>
+        <v>2845</v>
       </c>
       <c r="X18" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,1,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,2,1)),Transactions!$E$5:$E$1004)</f>
@@ -2916,7 +2994,7 @@
       </c>
       <c r="Y18" s="6">
         <f t="shared" ref="Y18:Y29" si="0">W18-X18</f>
-        <v>622.6</v>
+        <v>2017.6</v>
       </c>
     </row>
     <row r="19" spans="22:25" x14ac:dyDescent="0.35">
@@ -2925,15 +3003,15 @@
       </c>
       <c r="W19" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,2,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,3,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X19" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,2,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,3,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>1662.4</v>
       </c>
       <c r="Y19" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1182.5999999999999</v>
       </c>
     </row>
     <row r="20" spans="22:25" x14ac:dyDescent="0.35">
@@ -2942,15 +3020,15 @@
       </c>
       <c r="W20" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,3,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,4,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X20" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,3,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,4,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="Y20" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
     </row>
     <row r="21" spans="22:25" x14ac:dyDescent="0.35">
@@ -2959,15 +3037,15 @@
       </c>
       <c r="W21" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,4,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,5,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X21" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,4,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,5,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2037.4</v>
       </c>
       <c r="Y21" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>807.59999999999991</v>
       </c>
     </row>
     <row r="22" spans="22:25" x14ac:dyDescent="0.35">
@@ -2976,15 +3054,15 @@
       </c>
       <c r="W22" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,5,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,6,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X22" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,5,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,6,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="Y22" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
     </row>
     <row r="23" spans="22:25" x14ac:dyDescent="0.35">
@@ -2993,15 +3071,15 @@
       </c>
       <c r="W23" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,6,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,7,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X23" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,6,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,7,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="Y23" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
     </row>
     <row r="24" spans="22:25" x14ac:dyDescent="0.35">
@@ -3010,15 +3088,15 @@
       </c>
       <c r="W24" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,7,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,8,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X24" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,7,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,8,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="Y24" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
     </row>
     <row r="25" spans="22:25" x14ac:dyDescent="0.35">
@@ -3027,15 +3105,15 @@
       </c>
       <c r="W25" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,8,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,9,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X25" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,8,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,9,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="Y25" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
     </row>
     <row r="26" spans="22:25" x14ac:dyDescent="0.35">
@@ -3044,15 +3122,15 @@
       </c>
       <c r="W26" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,9,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,10,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X26" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,9,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,10,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="Y26" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
     </row>
     <row r="27" spans="22:25" x14ac:dyDescent="0.35">
@@ -3061,15 +3139,15 @@
       </c>
       <c r="W27" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,10,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,11,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="X27" s="6">
         <f>SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE('Schedule E Summary'!$C$3,10,1))*(Transactions!$A$5:$A$1004&lt;DATE('Schedule E Summary'!$C$3,11,1)),Transactions!$E$5:$E$1004)</f>
-        <v>0</v>
+        <v>2037.4</v>
       </c>
       <c r="Y27" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>807.59999999999991</v>
       </c>
     </row>
     <row r="28" spans="22:25" x14ac:dyDescent="0.35">
@@ -3180,11 +3258,11 @@
       </c>
       <c r="W38" s="6">
         <f>'Schedule E Summary'!M12</f>
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="X38">
         <f>W38+96/1000000</f>
-        <v>9.6000000000000002E-5</v>
+        <v>1050.000096</v>
       </c>
     </row>
     <row r="39" spans="22:24" x14ac:dyDescent="0.35">
@@ -3222,11 +3300,11 @@
       </c>
       <c r="W41" s="6">
         <f>'Schedule E Summary'!M15</f>
-        <v>612.4</v>
+        <v>6123.9999999999991</v>
       </c>
       <c r="X41">
         <f>W41+93/1000000</f>
-        <v>612.40009299999997</v>
+        <v>6124.0000929999987</v>
       </c>
     </row>
     <row r="42" spans="22:24" x14ac:dyDescent="0.35">
@@ -3278,11 +3356,11 @@
       </c>
       <c r="W45" s="6">
         <f>'Schedule E Summary'!M19</f>
-        <v>0</v>
+        <v>2850</v>
       </c>
       <c r="X45">
         <f>W45+89/1000000</f>
-        <v>8.8999999999999995E-5</v>
+        <v>2850.0000890000001</v>
       </c>
     </row>
     <row r="46" spans="22:24" x14ac:dyDescent="0.35">
@@ -3352,37 +3430,37 @@
       </c>
       <c r="W54" s="6">
         <f>IF(LARGE($X$34:$X$48,2)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,2),2))</f>
-        <v>612.4</v>
+        <v>6124</v>
       </c>
     </row>
     <row r="55" spans="22:23" x14ac:dyDescent="0.35">
       <c r="V55" t="str">
         <f>IF(LARGE($X$34:$X$48,3)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,3),$X$34:$X$48,0)))</f>
-        <v>Repairs</v>
+        <v>Taxes</v>
       </c>
       <c r="W55" s="6">
         <f>IF(LARGE($X$34:$X$48,3)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,3),2))</f>
-        <v>215</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="56" spans="22:23" x14ac:dyDescent="0.35">
       <c r="V56" t="str">
         <f>IF(LARGE($X$34:$X$48,4)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,4),$X$34:$X$48,0)))</f>
-        <v/>
+        <v>Insurance</v>
       </c>
       <c r="W56" s="6">
         <f>IF(LARGE($X$34:$X$48,4)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,4),2))</f>
-        <v>0</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="57" spans="22:23" x14ac:dyDescent="0.35">
       <c r="V57" t="str">
         <f>IF(LARGE($X$34:$X$48,5)&lt;0.01,"",INDEX($V$34:$V$48,MATCH(LARGE($X$34:$X$48,5),$X$34:$X$48,0)))</f>
-        <v/>
+        <v>Repairs</v>
       </c>
       <c r="W57" s="6">
         <f>IF(LARGE($X$34:$X$48,5)&lt;0.01,0,ROUND(LARGE($X$34:$X$48,5),2))</f>
-        <v>0</v>
+        <v>215</v>
       </c>
     </row>
     <row r="58" spans="22:23" x14ac:dyDescent="0.35">
@@ -3430,7 +3508,7 @@
       </c>
       <c r="W63" s="6">
         <f>IF(LARGE($X$5:$X$14,1)&lt;-100000000000,0,ROUND(LARGE($X$5:$X$14,1),2))</f>
-        <v>-7559.22</v>
+        <v>10029.18</v>
       </c>
     </row>
     <row r="64" spans="22:23" x14ac:dyDescent="0.35">
@@ -3931,7 +4009,7 @@
         <v>74</v>
       </c>
       <c r="E5" s="11">
-        <v>1450</v>
+        <v>2845</v>
       </c>
       <c r="F5" s="8" t="str">
         <f>IF(C5="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C5,Lists!$A$2:$A$17,0)),"?"))</f>
@@ -3961,7 +4039,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
-        <v>46053</v>
+        <v>46050</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>63</v>
@@ -3981,234 +4059,444 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="10"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
+      <c r="A8" s="10">
+        <v>46054</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="11">
+        <v>2845</v>
+      </c>
       <c r="F8" s="8" t="str">
         <f>IF(C8="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C8,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="11"/>
+      <c r="A9" s="10">
+        <v>46063</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="11">
+        <v>1050</v>
+      </c>
       <c r="F9" s="8" t="str">
         <f>IF(C9="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C9,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="10"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="11"/>
+      <c r="A10" s="10">
+        <v>46081</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F10" s="8" t="str">
         <f>IF(C10="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C10,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="10"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="11"/>
+      <c r="A11" s="10">
+        <v>46082</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="11">
+        <v>2845</v>
+      </c>
       <c r="F11" s="8" t="str">
         <f>IF(C11="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C11,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="11"/>
+      <c r="A12" s="10">
+        <v>46109</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F12" s="8" t="str">
         <f>IF(C12="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C12,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="10"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="11"/>
+      <c r="A13" s="10">
+        <v>46113</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="11">
+        <v>2845</v>
+      </c>
       <c r="F13" s="8" t="str">
         <f>IF(C13="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C13,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="10"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="11"/>
+      <c r="A14" s="10">
+        <v>46122</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="11">
+        <v>1425</v>
+      </c>
       <c r="F14" s="8" t="str">
         <f>IF(C14="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C14,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="10"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="11"/>
+      <c r="A15" s="10">
+        <v>46140</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F15" s="8" t="str">
         <f>IF(C15="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C15,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="10"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="11"/>
+      <c r="A16" s="10">
+        <v>46143</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="11">
+        <v>2845</v>
+      </c>
       <c r="F16" s="8" t="str">
         <f>IF(C16="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C16,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="10"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="11"/>
+      <c r="A17" s="10">
+        <v>46170</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F17" s="8" t="str">
         <f>IF(C17="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C17,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="10"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="11"/>
+      <c r="A18" s="10">
+        <v>46174</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="11">
+        <v>2845</v>
+      </c>
       <c r="F18" s="8" t="str">
         <f>IF(C18="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C18,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="10"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="11"/>
+      <c r="A19" s="10">
+        <v>46201</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F19" s="8" t="str">
         <f>IF(C19="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C19,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="10"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="11"/>
+      <c r="A20" s="10">
+        <v>46204</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="11">
+        <v>2845</v>
+      </c>
       <c r="F20" s="8" t="str">
         <f>IF(C20="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C20,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="10"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="11"/>
+      <c r="A21" s="10">
+        <v>46231</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F21" s="8" t="str">
         <f>IF(C21="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C21,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="10"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="11"/>
+      <c r="A22" s="10">
+        <v>46235</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" s="11">
+        <v>2845</v>
+      </c>
       <c r="F22" s="8" t="str">
         <f>IF(C22="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C22,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="10"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="11"/>
+      <c r="A23" s="10">
+        <v>46262</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F23" s="8" t="str">
         <f>IF(C23="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C23,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="10"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="11"/>
+      <c r="A24" s="10">
+        <v>46266</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24" s="11">
+        <v>2845</v>
+      </c>
       <c r="F24" s="8" t="str">
         <f>IF(C24="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C24,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="10"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="11"/>
+      <c r="A25" s="10">
+        <v>46293</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F25" s="8" t="str">
         <f>IF(C25="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C25,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="10"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="11"/>
+      <c r="A26" s="10">
+        <v>46296</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" s="11">
+        <v>2845</v>
+      </c>
       <c r="F26" s="8" t="str">
         <f>IF(C26="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C26,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Income</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="10"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="11"/>
+      <c r="A27" s="10">
+        <v>46305</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" s="11">
+        <v>1425</v>
+      </c>
       <c r="F27" s="8" t="str">
         <f>IF(C27="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C27,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="10"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="11"/>
+      <c r="A28" s="10">
+        <v>46323</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E28" s="11">
+        <v>612.4</v>
+      </c>
       <c r="F28" s="8" t="str">
         <f>IF(C28="","",IFERROR(INDEX(Lists!$C$2:$C$17,MATCH(C28,Lists!$A$2:$A$17,0)),"?"))</f>
-        <v/>
+        <v>Expense</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
@@ -15037,23 +15325,23 @@
   <sheetData>
     <row r="1" spans="1:13" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="14" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="C3" s="15">
         <v>2026</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>70</v>
@@ -15099,19 +15387,19 @@
         <v>Property 10</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>73</v>
       </c>
       <c r="C6" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B6,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
-        <v>1450</v>
+        <v>28450</v>
       </c>
       <c r="D6" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B6,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15151,15 +15439,15 @@
       </c>
       <c r="M6" s="18">
         <f t="shared" ref="M6:M22" si="0">SUM(C6:L6)</f>
-        <v>1450</v>
+        <v>28450</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="C7" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B7,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15208,10 +15496,10 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="C8" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B8,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15260,10 +15548,10 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="C9" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B9,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15312,10 +15600,10 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="C10" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B10,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15364,10 +15652,10 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C11" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B11,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15416,14 +15704,14 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="C12" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B12,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="D12" s="17">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B12,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15463,15 +15751,15 @@
       </c>
       <c r="M12" s="18">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="C13" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B13,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15520,10 +15808,10 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="16" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="C14" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B14,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15572,14 +15860,14 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B15,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
-        <v>612.4</v>
+        <v>6123.9999999999991</v>
       </c>
       <c r="D15" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B15,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15619,15 +15907,15 @@
       </c>
       <c r="M15" s="20">
         <f t="shared" si="0"/>
-        <v>612.4</v>
+        <v>6123.9999999999991</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="C16" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B16,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15676,7 +15964,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>75</v>
@@ -15728,10 +16016,10 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C18" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B18,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15780,14 +16068,14 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="C19" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B19,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
-        <v>0</v>
+        <v>2850</v>
       </c>
       <c r="D19" s="19">
         <f>IF(Properties!$B$6="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$6,Transactions!$C$5:$C$1004,$B19,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15827,15 +16115,15 @@
       </c>
       <c r="M19" s="20">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="16" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="C20" s="17">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B20,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15884,10 +16172,10 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="C21" s="19">
         <f>IF(Properties!$B$5="",0,SUMIFS(Transactions!$E$5:$E$1004,Transactions!$B$5:$B$1004,Properties!$B$5,Transactions!$C$5:$C$1004,$B21,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1)))</f>
@@ -15936,10 +16224,10 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="C22" s="21">
         <f>Properties!I5</f>
@@ -15988,11 +16276,11 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B24" s="14" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="C24" s="20">
         <f t="shared" ref="C24:M24" si="1">C6+C7</f>
-        <v>1450</v>
+        <v>28450</v>
       </c>
       <c r="D24" s="20">
         <f t="shared" si="1"/>
@@ -16032,16 +16320,16 @@
       </c>
       <c r="M24" s="20">
         <f t="shared" si="1"/>
-        <v>1450</v>
+        <v>28450</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B25" s="14" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="C25" s="20">
         <f t="shared" ref="C25:M25" si="2">C8+C9+C10+C11+C12+C13+C14+C15+C16+C17+C18+C19+C20+C21+C22</f>
-        <v>9009.2181818181816</v>
+        <v>18420.818181818184</v>
       </c>
       <c r="D25" s="20">
         <f t="shared" si="2"/>
@@ -16081,16 +16369,16 @@
       </c>
       <c r="M25" s="20">
         <f t="shared" si="2"/>
-        <v>9009.2181818181816</v>
+        <v>18420.818181818184</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B26" s="22" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="C26" s="23">
         <f t="shared" ref="C26:M26" si="3">C24-C25</f>
-        <v>-7559.2181818181816</v>
+        <v>10029.181818181816</v>
       </c>
       <c r="D26" s="23">
         <f t="shared" si="3"/>
@@ -16130,12 +16418,12 @@
       </c>
       <c r="M26" s="23">
         <f t="shared" si="3"/>
-        <v>-7559.2181818181816</v>
+        <v>10029.181818181816</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B28" s="5" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="C28" s="24">
         <f>SUMIFS(Transactions!$E$5:$E$1004,Transactions!$A$5:$A$1004,"&gt;="&amp;DATE($C$3,1,1),Transactions!$A$5:$A$1004,"&lt;"&amp;DATE($C$3+1,1,1))-SUM(M6:M21)</f>
@@ -16144,12 +16432,12 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B29" s="5" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="C30" s="13">
         <f>Transactions!I2</f>
@@ -16183,20 +16471,20 @@
   <sheetData>
     <row r="1" spans="1:6" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3" s="14" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B4" s="14" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="C4" s="26">
         <f>'Schedule E Summary'!C3</f>
@@ -16217,7 +16505,7 @@
         <v>35</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -16226,7 +16514,7 @@
       </c>
       <c r="C7" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,1,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,2,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,1,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,2,1)),Transactions!$E$5:$E$1004))</f>
-        <v>1450</v>
+        <v>2845</v>
       </c>
       <c r="D7" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,1,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,2,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,1,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,2,1)),Transactions!$E$5:$E$1004))</f>
@@ -16234,11 +16522,11 @@
       </c>
       <c r="E7" s="12">
         <f t="shared" ref="E7:E18" si="0">C7-D7</f>
-        <v>622.6</v>
+        <v>2017.6</v>
       </c>
       <c r="F7" s="12">
         <f>SUM($E$7:E7)</f>
-        <v>622.6</v>
+        <v>2017.6</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -16247,19 +16535,19 @@
       </c>
       <c r="C8" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,2,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,3,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,2,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,3,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D8" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,2,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,3,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,2,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,3,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>1662.4</v>
       </c>
       <c r="E8" s="29">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1182.5999999999999</v>
       </c>
       <c r="F8" s="29">
         <f>SUM($E$7:E8)</f>
-        <v>622.6</v>
+        <v>3200.2</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -16268,19 +16556,19 @@
       </c>
       <c r="C9" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,3,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,4,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,3,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,4,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D9" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,3,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,4,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,3,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,4,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="E9" s="12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
       <c r="F9" s="12">
         <f>SUM($E$7:E9)</f>
-        <v>622.6</v>
+        <v>5432.7999999999993</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -16289,19 +16577,19 @@
       </c>
       <c r="C10" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,4,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,5,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,4,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,5,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D10" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,4,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,5,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,4,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,5,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2037.4</v>
       </c>
       <c r="E10" s="29">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>807.59999999999991</v>
       </c>
       <c r="F10" s="29">
         <f>SUM($E$7:E10)</f>
-        <v>622.6</v>
+        <v>6240.4</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -16310,19 +16598,19 @@
       </c>
       <c r="C11" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,5,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,6,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,5,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,6,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D11" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,5,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,6,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,5,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,6,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="E11" s="12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
       <c r="F11" s="12">
         <f>SUM($E$7:E11)</f>
-        <v>622.6</v>
+        <v>8473</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
@@ -16331,19 +16619,19 @@
       </c>
       <c r="C12" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,6,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,7,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,6,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,7,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D12" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,6,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,7,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,6,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,7,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="E12" s="29">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
       <c r="F12" s="29">
         <f>SUM($E$7:E12)</f>
-        <v>622.6</v>
+        <v>10705.6</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
@@ -16352,19 +16640,19 @@
       </c>
       <c r="C13" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,7,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,8,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,7,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,8,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D13" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,7,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,8,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,7,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,8,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="E13" s="12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
       <c r="F13" s="12">
         <f>SUM($E$7:E13)</f>
-        <v>622.6</v>
+        <v>12938.2</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
@@ -16373,19 +16661,19 @@
       </c>
       <c r="C14" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,8,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,9,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,8,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,9,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D14" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,8,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,9,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,8,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,9,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="E14" s="29">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
       <c r="F14" s="29">
         <f>SUM($E$7:E14)</f>
-        <v>622.6</v>
+        <v>15170.800000000001</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
@@ -16394,19 +16682,19 @@
       </c>
       <c r="C15" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,9,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,10,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,9,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,10,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D15" s="12">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,9,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,10,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,9,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,10,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>612.4</v>
       </c>
       <c r="E15" s="12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2232.6</v>
       </c>
       <c r="F15" s="12">
         <f>SUM($E$7:E15)</f>
-        <v>622.6</v>
+        <v>17403.400000000001</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -16415,19 +16703,19 @@
       </c>
       <c r="C16" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,10,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,11,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$2:$A$3,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,10,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,11,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2845</v>
       </c>
       <c r="D16" s="29">
         <f>IF($C$3="All properties",SUMPRODUCT(ISNUMBER(MATCH(Transactions!$B$5:$B$1004,Lists!$F$3:$F$12,0))*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,10,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,11,1)),Transactions!$E$5:$E$1004),SUMPRODUCT((Transactions!$B$5:$B$1004=$C$3)*ISNUMBER(MATCH(Transactions!$C$5:$C$1004,Lists!$A$4:$A$17,0))*ISNUMBER(Transactions!$A$5:$A$1004)*(Transactions!$A$5:$A$1004&gt;=DATE($C$4,10,1))*(Transactions!$A$5:$A$1004&lt;DATE($C$4,11,1)),Transactions!$E$5:$E$1004))</f>
-        <v>0</v>
+        <v>2037.4</v>
       </c>
       <c r="E16" s="29">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>807.59999999999991</v>
       </c>
       <c r="F16" s="29">
         <f>SUM($E$7:E16)</f>
-        <v>622.6</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.35">
@@ -16448,7 +16736,7 @@
       </c>
       <c r="F17" s="12">
         <f>SUM($E$7:E17)</f>
-        <v>622.6</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.35">
@@ -16469,29 +16757,29 @@
       </c>
       <c r="F18" s="29">
         <f>SUM($E$7:E18)</f>
-        <v>622.6</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="14" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="C19" s="20">
         <f>SUM(C7:C18)</f>
-        <v>1450</v>
+        <v>28450</v>
       </c>
       <c r="D19" s="20">
         <f>SUM(D7:D18)</f>
-        <v>827.4</v>
+        <v>10238.999999999998</v>
       </c>
       <c r="E19" s="20">
         <f>SUM(E7:E18)</f>
-        <v>622.6</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -16531,12 +16819,12 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -16544,28 +16832,28 @@
         <v>26</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -16573,13 +16861,13 @@
         <v>63</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="E5" s="11">
         <v>1450</v>
@@ -16595,21 +16883,37 @@
       </c>
       <c r="I5" s="27">
         <f t="shared" ref="I5:I36" ca="1" si="0">IF(H5="","",IFERROR(H5-TODAY(),"check date"))</f>
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="27" t="str">
+      <c r="A6" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="E6" s="11">
+        <v>1395</v>
+      </c>
+      <c r="F6" s="11">
+        <v>1395</v>
+      </c>
+      <c r="G6" s="10">
+        <v>46082</v>
+      </c>
+      <c r="H6" s="10">
+        <v>46446</v>
+      </c>
+      <c r="I6" s="27">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -17426,11 +17730,11 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="14" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="E66" s="20">
         <f>SUM(E5:E64)</f>
-        <v>1450</v>
+        <v>2845</v>
       </c>
     </row>
   </sheetData>
@@ -17471,16 +17775,16 @@
         <v>70</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="C1" t="s">
         <v>72</v>
       </c>
       <c r="E1" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="H1" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
@@ -17488,30 +17792,30 @@
         <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="H2" t="s">
         <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>
@@ -17525,57 +17829,57 @@
         <v>EXAMPLE: 412 Maple St (duplex)</v>
       </c>
       <c r="H3" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="I3" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="J3" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="K3" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="L3" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="M3" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="N3" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="O3" t="s">
         <v>77</v>
       </c>
       <c r="P3" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="Q3" t="s">
         <v>75</v>
       </c>
       <c r="R3" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="S3" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="T3" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="U3" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="C4" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E4" t="str">
         <f>IF(Properties!B6="","",Properties!B6)</f>
@@ -17588,13 +17892,13 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="C5" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E5" t="str">
         <f>IF(Properties!B7="","",Properties!B7)</f>
@@ -17607,13 +17911,13 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E6" t="str">
         <f>IF(Properties!B8="","",Properties!B8)</f>
@@ -17626,13 +17930,13 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="C7" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E7" t="str">
         <f>IF(Properties!B9="","",Properties!B9)</f>
@@ -17645,13 +17949,13 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E8" t="str">
         <f>IF(Properties!B10="","",Properties!B10)</f>
@@ -17664,13 +17968,13 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="C9" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E9" t="str">
         <f>IF(Properties!B11="","",Properties!B11)</f>
@@ -17683,13 +17987,13 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="B10" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E10" t="str">
         <f>IF(Properties!B12="","",Properties!B12)</f>
@@ -17705,10 +18009,10 @@
         <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="C11" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E11" t="str">
         <f>IF(Properties!B13="","",Properties!B13)</f>
@@ -17721,13 +18025,13 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="C12" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="E12" t="str">
         <f>IF(Properties!B14="","",Properties!B14)</f>
@@ -17743,54 +18047,54 @@
         <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="C13" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="C14" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="C15" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="C16" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="C17" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>